<commit_message>
actualizacion de plantilla reporte quincenal
</commit_message>
<xml_diff>
--- a/backend/plantillas/plantilla_quincenal.xlsx
+++ b/backend/plantillas/plantilla_quincenal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesssemujeres/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesssemujeres/Desktop/sistema-rh/backend/plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F98C1868-3045-674C-9F0C-D06E1BAE3089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02BE0F92-620A-0C4E-A255-0245B5D42F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8780" yWindow="4180" windowWidth="32220" windowHeight="18060" xr2:uid="{27937616-F473-E74D-B3DC-537215079466}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="7">
   <si>
     <t>NUM DE EMPLEADO</t>
   </si>
@@ -141,13 +141,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500AB4D1-D5F2-9249-AE3C-08CDC7B95831}">
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" style="1" customWidth="1"/>
@@ -497,120 +497,126 @@
     <col min="4" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:35" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:33" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:35" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="T3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="U3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="V3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="W3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="X3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="Z3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="AB3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="AD3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="AF3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG3" s="6" t="s">
+      <c r="D3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AB3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AF3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="AH3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="AI3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
+    <row r="4" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
       <c r="C4" s="5"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
@@ -642,27 +648,30 @@
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
       <c r="AG4" s="5"/>
+      <c r="AH4" s="5"/>
+      <c r="AI4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
+  <mergeCells count="19">
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
+    <mergeCell ref="X4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="R4:S4"/>
     <mergeCell ref="T4:U4"/>
     <mergeCell ref="V4:W4"/>
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="L4:M4"/>
     <mergeCell ref="N4:O4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
correccion descarga de plantilla
</commit_message>
<xml_diff>
--- a/backend/plantillas/plantilla_quincenal.xlsx
+++ b/backend/plantillas/plantilla_quincenal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesssemujeres/Desktop/sistema-rh/backend/plantillas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesssemujeres/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02BE0F92-620A-0C4E-A255-0245B5D42F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130A1284-8C5C-8E43-AB03-2417805CC7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8780" yWindow="4180" windowWidth="32220" windowHeight="18060" xr2:uid="{27937616-F473-E74D-B3DC-537215079466}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="7">
   <si>
     <t>NUM DE EMPLEADO</t>
   </si>
@@ -488,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{500AB4D1-D5F2-9249-AE3C-08CDC7B95831}">
-  <dimension ref="A1:AI4"/>
+  <dimension ref="A1:AG4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" style="1" customWidth="1"/>
@@ -497,17 +497,17 @@
     <col min="4" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:33" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:33" s="3" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -607,14 +607,8 @@
       <c r="AG3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="AH3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI3" s="4" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="4" spans="1:35" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:33" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="5"/>
@@ -648,16 +642,9 @@
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
       <c r="AG4" s="5"/>
-      <c r="AH4" s="5"/>
-      <c r="AI4" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AH4:AI4"/>
+  <mergeCells count="18">
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="R4:S4"/>
@@ -669,6 +656,10 @@
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="L4:M4"/>
     <mergeCell ref="N4:O4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="X4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AD4:AE4"/>
     <mergeCell ref="AF4:AG4"/>

</xml_diff>

<commit_message>
modifcaciones colores en sabana y excel descargable
</commit_message>
<xml_diff>
--- a/backend/plantillas/plantilla_quincenal.xlsx
+++ b/backend/plantillas/plantilla_quincenal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesssemujeres/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{895B05C2-E1E0-6941-983C-016F43A87199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CED262-C3A5-5A4A-84CD-02A92BE9EED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8780" yWindow="4180" windowWidth="32220" windowHeight="18060" xr2:uid="{27937616-F473-E74D-B3DC-537215079466}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -75,34 +75,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color theme="0"/>
-      <name val="CalibrI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
+      <sz val="7"/>
       <color theme="1"/>
       <name val="CalibrI"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
-      <sz val="8"/>
+      <sz val="7"/>
       <color theme="0"/>
-      <name val="CalibrI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="CalibrI"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color theme="1"/>
       <name val="CalibrI"/>
       <family val="2"/>
     </font>
@@ -215,55 +196,46 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -607,195 +579,134 @@
   <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="29.33203125" style="16" customWidth="1"/>
-    <col min="3" max="3" width="36.33203125" style="6" customWidth="1"/>
-    <col min="4" max="33" width="7.6640625" style="7" customWidth="1"/>
-    <col min="34" max="36" width="10.83203125" style="5"/>
-    <col min="37" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="6.6640625" style="12" customWidth="1"/>
+    <col min="2" max="2" width="17.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="19.5" style="2" customWidth="1"/>
+    <col min="4" max="36" width="7.6640625" style="12" customWidth="1"/>
+    <col min="37" max="16384" width="10.83203125" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:36" s="5" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
-      <c r="AF1" s="4"/>
-      <c r="AG1" s="4"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="4"/>
     </row>
-    <row r="2" spans="1:36" s="1" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:36" s="5" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
-      <c r="Y2" s="4"/>
-      <c r="Z2" s="4"/>
-      <c r="AA2" s="4"/>
-      <c r="AB2" s="4"/>
-      <c r="AC2" s="4"/>
-      <c r="AD2" s="4"/>
-      <c r="AE2" s="4"/>
-      <c r="AF2" s="4"/>
-      <c r="AG2" s="4"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:36" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:36" s="5" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="S3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="T3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="U3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="W3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="X3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="Y3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="AA3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="AC3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="AE3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="AG3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH3" s="10"/>
-      <c r="AI3" s="10"/>
-      <c r="AJ3" s="10"/>
+      <c r="D3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="R3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="S3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="T3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="U3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="V3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="Y3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="AC3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="6"/>
+      <c r="AJ3" s="6"/>
     </row>
-    <row r="4" spans="1:36" s="1" customFormat="1" ht="12" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
+    <row r="4" spans="1:36" s="5" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
@@ -827,17 +738,12 @@
       <c r="AE4" s="11"/>
       <c r="AF4" s="11"/>
       <c r="AG4" s="11"/>
-      <c r="AH4" s="11"/>
-      <c r="AI4" s="11"/>
-      <c r="AJ4" s="11"/>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="10"/>
+      <c r="AJ4" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="X4:Y4"/>
-    <mergeCell ref="Z4:AA4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
     <mergeCell ref="AH3:AH4"/>
     <mergeCell ref="AI3:AI4"/>
     <mergeCell ref="AJ3:AJ4"/>
@@ -854,6 +760,11 @@
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
+    <mergeCell ref="X4:Y4"/>
+    <mergeCell ref="Z4:AA4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>